<commit_message>
chore(weekly-sync): auto-pull through 2026-08-03
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Audio_Array/ads_report_week31.xlsx
+++ b/data/ams_weekly_data/Audio_Array/ads_report_week31.xlsx
@@ -1,14 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SP" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SD" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SP" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="SD" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SB" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,16 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +36,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +44,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,42 +419,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Portfolio name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Campaign Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Advertised ASIN</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Clicks</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>14 Day Total Sales (₹)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>14 Day Total Units (#)</t>
         </is>
@@ -512,13 +501,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>701.35</v>
+        <v>692.77</v>
       </c>
       <c r="E3" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F3" t="n">
-        <v>8065</v>
+        <v>8060</v>
       </c>
       <c r="G3" t="n">
         <v>1280.51</v>
@@ -546,7 +535,7 @@
         <v>187</v>
       </c>
       <c r="F4" t="n">
-        <v>24632</v>
+        <v>24630</v>
       </c>
       <c r="G4" t="n">
         <v>3821.19</v>
@@ -630,13 +619,13 @@
         <v>209</v>
       </c>
       <c r="F7" t="n">
-        <v>9936</v>
+        <v>9934</v>
       </c>
       <c r="G7" t="n">
         <v>9401.67</v>
       </c>
       <c r="H7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -742,7 +731,7 @@
         <v>28</v>
       </c>
       <c r="F11" t="n">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="G11" t="n">
         <v>2202.54</v>
@@ -854,7 +843,7 @@
         <v>365</v>
       </c>
       <c r="F15" t="n">
-        <v>32303</v>
+        <v>32300</v>
       </c>
       <c r="G15" t="n">
         <v>21013.56</v>
@@ -941,10 +930,10 @@
         <v>56288</v>
       </c>
       <c r="G18" t="n">
-        <v>49456.8</v>
+        <v>47170.36</v>
       </c>
       <c r="H18" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="19">
@@ -1025,10 +1014,10 @@
         <v>6716</v>
       </c>
       <c r="G21" t="n">
-        <v>6266.95</v>
+        <v>7961.02</v>
       </c>
       <c r="H21" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22">
@@ -1302,7 +1291,7 @@
         <v>161</v>
       </c>
       <c r="F31" t="n">
-        <v>8506</v>
+        <v>8504</v>
       </c>
       <c r="G31" t="n">
         <v>16264.4</v>
@@ -1330,7 +1319,7 @@
         <v>1092</v>
       </c>
       <c r="F32" t="n">
-        <v>99457</v>
+        <v>99456</v>
       </c>
       <c r="G32" t="n">
         <v>56819.47</v>
@@ -1414,7 +1403,7 @@
         <v>340</v>
       </c>
       <c r="F35" t="n">
-        <v>63227</v>
+        <v>63225</v>
       </c>
       <c r="G35" t="n">
         <v>16136.46</v>
@@ -1464,13 +1453,13 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>2176.28</v>
+        <v>2159.8</v>
       </c>
       <c r="E37" t="n">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F37" t="n">
-        <v>25318</v>
+        <v>25317</v>
       </c>
       <c r="G37" t="n">
         <v>32027.94</v>
@@ -1694,7 +1683,7 @@
         <v>1125</v>
       </c>
       <c r="F45" t="n">
-        <v>148963</v>
+        <v>148959</v>
       </c>
       <c r="G45" t="n">
         <v>76812.71000000001</v>
@@ -1722,7 +1711,7 @@
         <v>180</v>
       </c>
       <c r="F46" t="n">
-        <v>27943</v>
+        <v>27942</v>
       </c>
       <c r="G46" t="n">
         <v>0</v>
@@ -1750,7 +1739,7 @@
         <v>454</v>
       </c>
       <c r="F47" t="n">
-        <v>86614</v>
+        <v>86613</v>
       </c>
       <c r="G47" t="n">
         <v>5088.98</v>
@@ -1834,7 +1823,7 @@
         <v>292</v>
       </c>
       <c r="F50" t="n">
-        <v>37564</v>
+        <v>37562</v>
       </c>
       <c r="G50" t="n">
         <v>6776.27</v>
@@ -1865,10 +1854,10 @@
         <v>53645</v>
       </c>
       <c r="G51" t="n">
-        <v>28027.92</v>
+        <v>30077.08</v>
       </c>
       <c r="H51" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="52">
@@ -2002,7 +1991,7 @@
         <v>1300</v>
       </c>
       <c r="F56" t="n">
-        <v>154804</v>
+        <v>154803</v>
       </c>
       <c r="G56" t="n">
         <v>69079.7</v>
@@ -2814,7 +2803,7 @@
         <v>41</v>
       </c>
       <c r="F85" t="n">
-        <v>16818</v>
+        <v>16817</v>
       </c>
       <c r="G85" t="n">
         <v>0</v>
@@ -2842,7 +2831,7 @@
         <v>86</v>
       </c>
       <c r="F86" t="n">
-        <v>7962</v>
+        <v>7961</v>
       </c>
       <c r="G86" t="n">
         <v>3999.15</v>
@@ -2926,7 +2915,7 @@
         <v>643</v>
       </c>
       <c r="F89" t="n">
-        <v>139795</v>
+        <v>139793</v>
       </c>
       <c r="G89" t="n">
         <v>33127.96</v>
@@ -2954,7 +2943,7 @@
         <v>152</v>
       </c>
       <c r="F90" t="n">
-        <v>9686</v>
+        <v>9685</v>
       </c>
       <c r="G90" t="n">
         <v>8384.719999999999</v>
@@ -2982,7 +2971,7 @@
         <v>81</v>
       </c>
       <c r="F91" t="n">
-        <v>18339</v>
+        <v>18337</v>
       </c>
       <c r="G91" t="n">
         <v>15174.58</v>
@@ -3013,10 +3002,10 @@
         <v>42812</v>
       </c>
       <c r="G92" t="n">
-        <v>13233.01</v>
+        <v>16646.57</v>
       </c>
       <c r="H92" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="93">
@@ -3066,7 +3055,7 @@
         <v>430</v>
       </c>
       <c r="F94" t="n">
-        <v>66915</v>
+        <v>66914</v>
       </c>
       <c r="G94" t="n">
         <v>27315.24</v>
@@ -3122,7 +3111,7 @@
         <v>955</v>
       </c>
       <c r="F96" t="n">
-        <v>106257</v>
+        <v>106254</v>
       </c>
       <c r="G96" t="n">
         <v>14060.16</v>
@@ -3150,7 +3139,7 @@
         <v>35</v>
       </c>
       <c r="F97" t="n">
-        <v>14595</v>
+        <v>14594</v>
       </c>
       <c r="G97" t="n">
         <v>1007.63</v>
@@ -3178,7 +3167,7 @@
         <v>14</v>
       </c>
       <c r="F98" t="n">
-        <v>3713</v>
+        <v>3712</v>
       </c>
       <c r="G98" t="n">
         <v>3982.2</v>
@@ -3234,7 +3223,7 @@
         <v>47</v>
       </c>
       <c r="F100" t="n">
-        <v>13004</v>
+        <v>13003</v>
       </c>
       <c r="G100" t="n">
         <v>0</v>
@@ -3262,7 +3251,7 @@
         <v>32</v>
       </c>
       <c r="F101" t="n">
-        <v>5326</v>
+        <v>5325</v>
       </c>
       <c r="G101" t="n">
         <v>3157.63</v>
@@ -3318,13 +3307,13 @@
         <v>47</v>
       </c>
       <c r="F103" t="n">
-        <v>7588</v>
+        <v>7587</v>
       </c>
       <c r="G103" t="n">
-        <v>3388.98</v>
+        <v>4744.06</v>
       </c>
       <c r="H103" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="104">
@@ -3458,7 +3447,7 @@
         <v>393</v>
       </c>
       <c r="F108" t="n">
-        <v>45390</v>
+        <v>45389</v>
       </c>
       <c r="G108" t="n">
         <v>4611.04</v>
@@ -3486,7 +3475,7 @@
         <v>9</v>
       </c>
       <c r="F109" t="n">
-        <v>1155</v>
+        <v>1154</v>
       </c>
       <c r="G109" t="n">
         <v>0</v>
@@ -3514,13 +3503,13 @@
         <v>2465</v>
       </c>
       <c r="F110" t="n">
-        <v>484754</v>
+        <v>484747</v>
       </c>
       <c r="G110" t="n">
-        <v>17299.14</v>
+        <v>18323.72</v>
       </c>
       <c r="H110" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="111">
@@ -3542,7 +3531,7 @@
         <v>610</v>
       </c>
       <c r="F111" t="n">
-        <v>102747</v>
+        <v>102745</v>
       </c>
       <c r="G111" t="n">
         <v>7368.65</v>
@@ -3570,7 +3559,7 @@
         <v>92</v>
       </c>
       <c r="F112" t="n">
-        <v>21658</v>
+        <v>21657</v>
       </c>
       <c r="G112" t="n">
         <v>3727.11</v>
@@ -3682,7 +3671,7 @@
         <v>158</v>
       </c>
       <c r="F116" t="n">
-        <v>16671</v>
+        <v>16670</v>
       </c>
       <c r="G116" t="n">
         <v>8005.92</v>
@@ -3906,7 +3895,7 @@
         <v>188</v>
       </c>
       <c r="F124" t="n">
-        <v>18677</v>
+        <v>18675</v>
       </c>
       <c r="G124" t="n">
         <v>12410.17</v>
@@ -3962,7 +3951,7 @@
         <v>192</v>
       </c>
       <c r="F126" t="n">
-        <v>30262</v>
+        <v>30261</v>
       </c>
       <c r="G126" t="n">
         <v>6795.75</v>
@@ -3990,7 +3979,7 @@
         <v>562</v>
       </c>
       <c r="F127" t="n">
-        <v>60048</v>
+        <v>60047</v>
       </c>
       <c r="G127" t="n">
         <v>8727.969999999999</v>
@@ -4046,7 +4035,7 @@
         <v>82</v>
       </c>
       <c r="F129" t="n">
-        <v>17244</v>
+        <v>17243</v>
       </c>
       <c r="G129" t="n">
         <v>0</v>
@@ -4158,13 +4147,13 @@
         <v>1235</v>
       </c>
       <c r="F133" t="n">
-        <v>135648</v>
+        <v>135647</v>
       </c>
       <c r="G133" t="n">
-        <v>10167.8</v>
+        <v>12455.09</v>
       </c>
       <c r="H133" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="134">
@@ -4410,7 +4399,7 @@
         <v>43</v>
       </c>
       <c r="F142" t="n">
-        <v>6267</v>
+        <v>6265</v>
       </c>
       <c r="G142" t="n">
         <v>0</v>
@@ -4469,10 +4458,10 @@
         <v>21483</v>
       </c>
       <c r="G144" t="n">
-        <v>5083.9</v>
+        <v>15546.61</v>
       </c>
       <c r="H144" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="145">
@@ -4718,7 +4707,7 @@
         <v>324</v>
       </c>
       <c r="F153" t="n">
-        <v>54963</v>
+        <v>54961</v>
       </c>
       <c r="G153" t="n">
         <v>8894.049999999999</v>
@@ -4805,10 +4794,10 @@
         <v>15871</v>
       </c>
       <c r="G156" t="n">
-        <v>6793.22</v>
+        <v>9058.470000000001</v>
       </c>
       <c r="H156" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="157">
@@ -4830,7 +4819,7 @@
         <v>108</v>
       </c>
       <c r="F157" t="n">
-        <v>20700</v>
+        <v>20699</v>
       </c>
       <c r="G157" t="n">
         <v>15249.18</v>
@@ -4942,7 +4931,7 @@
         <v>495</v>
       </c>
       <c r="F161" t="n">
-        <v>67614</v>
+        <v>67613</v>
       </c>
       <c r="G161" t="n">
         <v>21521.19</v>
@@ -5138,7 +5127,7 @@
         <v>159</v>
       </c>
       <c r="F168" t="n">
-        <v>26718</v>
+        <v>26717</v>
       </c>
       <c r="G168" t="n">
         <v>6528.82</v>
@@ -5194,7 +5183,7 @@
         <v>13</v>
       </c>
       <c r="F170" t="n">
-        <v>3112</v>
+        <v>3111</v>
       </c>
       <c r="G170" t="n">
         <v>0</v>
@@ -5362,7 +5351,7 @@
         <v>65</v>
       </c>
       <c r="F176" t="n">
-        <v>15307</v>
+        <v>15306</v>
       </c>
       <c r="G176" t="n">
         <v>2965.25</v>
@@ -5390,7 +5379,7 @@
         <v>190</v>
       </c>
       <c r="F177" t="n">
-        <v>23292</v>
+        <v>23290</v>
       </c>
       <c r="G177" t="n">
         <v>12744.07</v>
@@ -5925,10 +5914,10 @@
         <v>37304</v>
       </c>
       <c r="G196" t="n">
-        <v>7981.370000000001</v>
+        <v>11224.59</v>
       </c>
       <c r="H196" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="197">
@@ -5981,10 +5970,10 @@
         <v>7188</v>
       </c>
       <c r="G198" t="n">
-        <v>2795.76</v>
+        <v>5082.200000000001</v>
       </c>
       <c r="H198" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="199">
@@ -6006,7 +5995,7 @@
         <v>103</v>
       </c>
       <c r="F199" t="n">
-        <v>81394</v>
+        <v>81392</v>
       </c>
       <c r="G199" t="n">
         <v>4828.809999999999</v>
@@ -6062,7 +6051,7 @@
         <v>93</v>
       </c>
       <c r="F201" t="n">
-        <v>101879</v>
+        <v>101876</v>
       </c>
       <c r="G201" t="n">
         <v>2117.8</v>
@@ -6622,7 +6611,7 @@
         <v>47</v>
       </c>
       <c r="F221" t="n">
-        <v>6027</v>
+        <v>6025</v>
       </c>
       <c r="G221" t="n">
         <v>2032.2</v>
@@ -6672,13 +6661,13 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>810.8199999999999</v>
+        <v>805.37</v>
       </c>
       <c r="E223" t="n">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F223" t="n">
-        <v>50742</v>
+        <v>50741</v>
       </c>
       <c r="G223" t="n">
         <v>6437.28</v>
@@ -6818,13 +6807,13 @@
         <v>203</v>
       </c>
       <c r="F228" t="n">
-        <v>37016</v>
+        <v>37015</v>
       </c>
       <c r="G228" t="n">
-        <v>5844.06</v>
+        <v>4234.74</v>
       </c>
       <c r="H228" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="229">
@@ -6986,13 +6975,13 @@
         <v>1117</v>
       </c>
       <c r="F234" t="n">
-        <v>123889</v>
+        <v>123887</v>
       </c>
       <c r="G234" t="n">
-        <v>76825.44</v>
+        <v>83684.75999999999</v>
       </c>
       <c r="H234" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="235">
@@ -7182,7 +7171,7 @@
         <v>15</v>
       </c>
       <c r="F241" t="n">
-        <v>1317</v>
+        <v>1316</v>
       </c>
       <c r="G241" t="n">
         <v>2879.66</v>
@@ -7350,7 +7339,7 @@
         <v>65</v>
       </c>
       <c r="F247" t="n">
-        <v>4813</v>
+        <v>4812</v>
       </c>
       <c r="G247" t="n">
         <v>4963.56</v>
@@ -7378,7 +7367,7 @@
         <v>405</v>
       </c>
       <c r="F248" t="n">
-        <v>43621</v>
+        <v>43617</v>
       </c>
       <c r="G248" t="n">
         <v>10294.91</v>
@@ -7406,13 +7395,13 @@
         <v>661</v>
       </c>
       <c r="F249" t="n">
-        <v>51213</v>
+        <v>51212</v>
       </c>
       <c r="G249" t="n">
-        <v>7626.27</v>
+        <v>12710.17</v>
       </c>
       <c r="H249" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="250">
@@ -7605,10 +7594,10 @@
         <v>18234</v>
       </c>
       <c r="G256" t="n">
-        <v>12730.51</v>
+        <v>15973.73</v>
       </c>
       <c r="H256" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="257">
@@ -7630,7 +7619,7 @@
         <v>84</v>
       </c>
       <c r="F257" t="n">
-        <v>19609</v>
+        <v>19607</v>
       </c>
       <c r="G257" t="n">
         <v>2117.8</v>
@@ -7661,10 +7650,10 @@
         <v>40238</v>
       </c>
       <c r="G258" t="n">
-        <v>13511.84</v>
+        <v>17249.97</v>
       </c>
       <c r="H258" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="259">
@@ -8050,7 +8039,7 @@
         <v>8</v>
       </c>
       <c r="F272" t="n">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="G272" t="n">
         <v>0</v>
@@ -8249,10 +8238,10 @@
         <v>3970</v>
       </c>
       <c r="G279" t="n">
-        <v>0</v>
+        <v>2286.44</v>
       </c>
       <c r="H279" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="280">
@@ -8414,7 +8403,7 @@
         <v>54</v>
       </c>
       <c r="F285" t="n">
-        <v>7521</v>
+        <v>7518</v>
       </c>
       <c r="G285" t="n">
         <v>5082.21</v>
@@ -8498,7 +8487,7 @@
         <v>284</v>
       </c>
       <c r="F288" t="n">
-        <v>25011</v>
+        <v>25009</v>
       </c>
       <c r="G288" t="n">
         <v>35333.9</v>
@@ -8526,7 +8515,7 @@
         <v>6</v>
       </c>
       <c r="F289" t="n">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="G289" t="n">
         <v>2965.26</v>
@@ -8582,7 +8571,7 @@
         <v>92</v>
       </c>
       <c r="F291" t="n">
-        <v>10282</v>
+        <v>10281</v>
       </c>
       <c r="G291" t="n">
         <v>0</v>
@@ -8722,7 +8711,7 @@
         <v>23</v>
       </c>
       <c r="F296" t="n">
-        <v>2077</v>
+        <v>2076</v>
       </c>
       <c r="G296" t="n">
         <v>5591.52</v>
@@ -8806,7 +8795,7 @@
         <v>127</v>
       </c>
       <c r="F299" t="n">
-        <v>9944</v>
+        <v>9943</v>
       </c>
       <c r="G299" t="n">
         <v>0</v>
@@ -8862,7 +8851,7 @@
         <v>77</v>
       </c>
       <c r="F301" t="n">
-        <v>10251</v>
+        <v>10248</v>
       </c>
       <c r="G301" t="n">
         <v>0</v>
@@ -9248,13 +9237,13 @@
         </is>
       </c>
       <c r="D315" t="n">
-        <v>2306.27</v>
+        <v>2302.89</v>
       </c>
       <c r="E315" t="n">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F315" t="n">
-        <v>29042</v>
+        <v>29038</v>
       </c>
       <c r="G315" t="n">
         <v>16516.97</v>
@@ -9282,13 +9271,13 @@
         <v>212</v>
       </c>
       <c r="F316" t="n">
-        <v>54806</v>
+        <v>54805</v>
       </c>
       <c r="G316" t="n">
-        <v>6437.28</v>
+        <v>8046.599999999999</v>
       </c>
       <c r="H316" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="317">
@@ -9338,7 +9327,7 @@
         <v>396</v>
       </c>
       <c r="F318" t="n">
-        <v>85581</v>
+        <v>85579</v>
       </c>
       <c r="G318" t="n">
         <v>3557.63</v>
@@ -9394,7 +9383,7 @@
         <v>130</v>
       </c>
       <c r="F320" t="n">
-        <v>20529</v>
+        <v>20528</v>
       </c>
       <c r="G320" t="n">
         <v>7284.75</v>
@@ -9534,7 +9523,7 @@
         <v>47</v>
       </c>
       <c r="F325" t="n">
-        <v>32237</v>
+        <v>32236</v>
       </c>
       <c r="G325" t="n">
         <v>1863.56</v>
@@ -9593,10 +9582,10 @@
         <v>17578</v>
       </c>
       <c r="G327" t="n">
-        <v>9827.120000000001</v>
+        <v>12283.9</v>
       </c>
       <c r="H327" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="328">
@@ -9674,7 +9663,7 @@
         <v>265</v>
       </c>
       <c r="F330" t="n">
-        <v>30568</v>
+        <v>30567</v>
       </c>
       <c r="G330" t="n">
         <v>3557.63</v>
@@ -9698,42 +9687,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Portfolio name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Campaign Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Advertised ASIN</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Clicks</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>14 Day Total Sales (₹)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>14 Day Total Units (#)</t>
         </is>
@@ -9898,7 +9887,7 @@
         <v>447</v>
       </c>
       <c r="F7" t="n">
-        <v>96468</v>
+        <v>96467</v>
       </c>
       <c r="G7" t="n">
         <v>15246.62</v>
@@ -9926,13 +9915,13 @@
         <v>338</v>
       </c>
       <c r="F8" t="n">
-        <v>96546</v>
+        <v>96545</v>
       </c>
       <c r="G8" t="n">
-        <v>8868.65</v>
+        <v>11537.29</v>
       </c>
       <c r="H8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -10097,10 +10086,10 @@
         <v>264877</v>
       </c>
       <c r="G14" t="n">
-        <v>62979.69</v>
+        <v>67075.45</v>
       </c>
       <c r="H14" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15">
@@ -10486,7 +10475,7 @@
         <v>924</v>
       </c>
       <c r="F28" t="n">
-        <v>169829</v>
+        <v>169827</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -10682,7 +10671,7 @@
         <v>581</v>
       </c>
       <c r="F35" t="n">
-        <v>120286</v>
+        <v>120285</v>
       </c>
       <c r="G35" t="n">
         <v>12761.02</v>
@@ -10732,10 +10721,10 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>413.55</v>
+        <v>411.91</v>
       </c>
       <c r="E37" t="n">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F37" t="n">
         <v>28979</v>
@@ -10816,19 +10805,19 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>4458.13</v>
+        <v>4454.18</v>
       </c>
       <c r="E40" t="n">
-        <v>3992</v>
+        <v>3987</v>
       </c>
       <c r="F40" t="n">
-        <v>663122</v>
+        <v>663112</v>
       </c>
       <c r="G40" t="n">
-        <v>31394.07</v>
+        <v>25038.99</v>
       </c>
       <c r="H40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="41">
@@ -10969,6 +10958,1222 @@
       </c>
       <c r="H45" t="n">
         <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Portfolio name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Campaign Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Advertised ASIN</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Impressions</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Clicks</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>14 Day Total Sales (₹)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>14 Day Total Units (#)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Audio Array-B0BPLZ5CGV-AI 04 Audio Interface-SBV -PT</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>B0BPLZ5CGV</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>14328</v>
+      </c>
+      <c r="E2" t="n">
+        <v>160</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1098.93</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Audio Array-B0CKHVHVQ1-AM W45 Wireless-SBV-KT-Phrase</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>B0CKHVHVQ1</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>77414</v>
+      </c>
+      <c r="E3" t="n">
+        <v>204</v>
+      </c>
+      <c r="F3" t="n">
+        <v>3069.87</v>
+      </c>
+      <c r="G3" t="n">
+        <v>9150.84</v>
+      </c>
+      <c r="H3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Audio Array-B0CKHVHVQ1-AM W45 Wireless-SBV-PT</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>B0CKHVHVQ1</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>68311</v>
+      </c>
+      <c r="E4" t="n">
+        <v>399</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2023.74</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>B0B4DPX2J2</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>339</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>B0B4DS678Q</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>339</v>
+      </c>
+      <c r="E6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>B0B4G19R58</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>339</v>
+      </c>
+      <c r="E7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>B0B4JRQP22</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>339</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>B0B4K87PR4</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>339</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>B0B4KC7VBM</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>339</v>
+      </c>
+      <c r="E10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>B0BLJVJ2GN</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>339</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>B0BLK8DNPD</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>339</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F12" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>B0BLNCP74M</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>5191</v>
+      </c>
+      <c r="E13" t="n">
+        <v>60</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1166.362378511303</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4815.419663719008</v>
+      </c>
+      <c r="H13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>B0BPLZ5CGV</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>339</v>
+      </c>
+      <c r="E14" t="n">
+        <v>3</v>
+      </c>
+      <c r="F14" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>B0C4YTNJG7</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>339</v>
+      </c>
+      <c r="E15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>B0C539RBGL</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>339</v>
+      </c>
+      <c r="E16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F16" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>B0CF5R3V95</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>339</v>
+      </c>
+      <c r="E17" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>B0CF5RRTDJ</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>339</v>
+      </c>
+      <c r="E18" t="n">
+        <v>3</v>
+      </c>
+      <c r="F18" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>B0CF5TCQKL</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>339</v>
+      </c>
+      <c r="E19" t="n">
+        <v>3</v>
+      </c>
+      <c r="F19" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>B0CH4RT4P8</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>339</v>
+      </c>
+      <c r="E20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F20" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>B0CKHVHVQ1</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>120565</v>
+      </c>
+      <c r="E21" t="n">
+        <v>500</v>
+      </c>
+      <c r="F21" t="n">
+        <v>4016.499629629629</v>
+      </c>
+      <c r="G21" t="n">
+        <v>12284.74</v>
+      </c>
+      <c r="H21" t="n">
+        <v>4</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>B0CM6NTWBP</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>339</v>
+      </c>
+      <c r="E22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F22" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>B0D3M1B4Z8</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>339</v>
+      </c>
+      <c r="E23" t="n">
+        <v>3</v>
+      </c>
+      <c r="F23" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>B0DFMLS8JG</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>339</v>
+      </c>
+      <c r="E24" t="n">
+        <v>3</v>
+      </c>
+      <c r="F24" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>B0DFMMTWLY</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>339</v>
+      </c>
+      <c r="E25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F25" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>B0DFMNGFTD</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>339</v>
+      </c>
+      <c r="E26" t="n">
+        <v>3</v>
+      </c>
+      <c r="F26" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>B0DT6T6N6B</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>339</v>
+      </c>
+      <c r="E27" t="n">
+        <v>3</v>
+      </c>
+      <c r="F27" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>B0FF9R3GKK</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>339</v>
+      </c>
+      <c r="E28" t="n">
+        <v>3</v>
+      </c>
+      <c r="F28" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>B0FJS57732</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>6725</v>
+      </c>
+      <c r="E29" t="n">
+        <v>78</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1511.127621488697</v>
+      </c>
+      <c r="G29" t="n">
+        <v>6238.810336280993</v>
+      </c>
+      <c r="H29" t="n">
+        <v>3</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>B0G2C2RCXN</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>339</v>
+      </c>
+      <c r="E30" t="n">
+        <v>3</v>
+      </c>
+      <c r="F30" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>B0G3Q517Y2</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>339</v>
+      </c>
+      <c r="E31" t="n">
+        <v>3</v>
+      </c>
+      <c r="F31" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>B0G3Q59X8C</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>339</v>
+      </c>
+      <c r="E32" t="n">
+        <v>3</v>
+      </c>
+      <c r="F32" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Audio Array-Multiple Ad Group-SB-PT</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>B0G4DNF8RZ</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>339</v>
+      </c>
+      <c r="E33" t="n">
+        <v>3</v>
+      </c>
+      <c r="F33" t="n">
+        <v>24.27962962962963</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Audio Array_B0DXFPM4N2_Studio Monitor_SB Video</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>B0DXFPM4N2</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>72781</v>
+      </c>
+      <c r="E34" t="n">
+        <v>579</v>
+      </c>
+      <c r="F34" t="n">
+        <v>3480.22</v>
+      </c>
+      <c r="G34" t="n">
+        <v>7626.27</v>
+      </c>
+      <c r="H34" t="n">
+        <v>2</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Audio Array_B0GKPXQ8G3_Wireless Mic_SBV</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>B0GKPXQ8G3</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>18095</v>
+      </c>
+      <c r="E35" t="n">
+        <v>131</v>
+      </c>
+      <c r="F35" t="n">
+        <v>1214.05</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Audio Array_Studio Headphones_SB_KT_Phrase</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>B0FG88HVQ8</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>44205</v>
+      </c>
+      <c r="E36" t="n">
+        <v>71</v>
+      </c>
+      <c r="F36" t="n">
+        <v>839.9400000000001</v>
+      </c>
+      <c r="G36" t="n">
+        <v>7961.869999999999</v>
+      </c>
+      <c r="H36" t="n">
+        <v>5</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Audio Array</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>